<commit_message>
Add Insights tab to school detail + My School nav for single-school roles
- school-detail: new Insights tab (Alongside AI summary), mirrors Alongside —
  visible to all personas, scope-filtered; default landing stays Visit allocation
- nav: My School entry for single-school roles (district keeps the Schools list);
  school-detail breadcrumb collapses for single-school personas
- reserve "Insights" for the Alongside AI view; TC analytics stay under Reports
- roles-matrix.xlsx: add "View Insights (Alongside AI summary)" row (all roles);
  relabel the Reports row to drop "insights"

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/roles-matrix.xlsx
+++ b/roles-matrix.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>roles-matrix.html</t>
+          <t>roles-matrix.html (retired — this xlsx is the source of truth)</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>View Reports (download insights)</t>
+          <t>View Reports (dashboards &amp; exports)</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -1657,51 +1657,51 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Library, reports &amp; insights</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>View Insights (Alongside AI summary)</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Mirrors Alongside Dashboard — all staff, data filtered by scope. School-scoped AI summary of student conversation themes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>System</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>System</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Student Demo (preview mode)</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E30" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F30" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G30" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>Sandboxed; no data writes.</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Self-Care mode (own private space)</t>
+          <t>Student Demo (preview mode)</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>Universal. Not visible to district.</t>
+          <t>Sandboxed; no data writes.</t>
         </is>
       </c>
     </row>
@@ -1755,35 +1755,77 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
+          <t>Self-Care mode (own private space)</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Universal. Not visible to district.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
           <t>Settings (own profile)</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F32" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G32" s="10" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>All users.</t>
         </is>
@@ -1792,7 +1834,7 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A30:H30"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A2:H2"/>

</xml_diff>